<commit_message>
Add activity audit logging system, operator context switcher, and Excel log worksheet
</commit_message>
<xml_diff>
--- a/Inventory_Ledger_Pachauri.xlsx
+++ b/Inventory_Ledger_Pachauri.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Inventory Ledger" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Activity Audit Log" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -687,7 +688,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Automated Inventory Tracking, Payment Reconciliation &amp; Balance Calculation</t>
+          <t>Automated Inventory Tracking, Payment Reconciliation &amp; Activity Audit Log</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2022,7 @@
       <c r="C68" s="4" t="n"/>
       <c r="E68" s="29" t="inlineStr">
         <is>
-          <t>5. Fill in 'Acknowledged By' and 'Date' columns whenever status is updated.</t>
+          <t>5. Every activity &amp; status update is automatically logged in the 'Activity Audit Log' tab!</t>
         </is>
       </c>
       <c r="F68" s="4" t="n"/>
@@ -2116,4 +2117,137 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PACHAURI INVENTORY ACTIVITY &amp; AUDIT TRAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Performed By (Operator)</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>Action Type</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>Activity Description &amp; Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-10 10:00:00</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>Dinesh Pachauri</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Item Added</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>Initial entry created: 7 inventory items added for Dinesh Pachauri (Total: ₹15,841.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-10 10:05:00</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Mukesh Pachauri</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Item Added</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Initial entry created: 6 inventory items added for Mukesh Pachauri (Total: ₹8,391.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-10 10:10:00</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>System Auto</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Ledger Generated</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Automated ledger initialized with net balance difference: Dinesh owes Mukesh ₹7,450.00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add PIN authentication modal, authorized user guards, and timestamped security audit logging
</commit_message>
<xml_diff>
--- a/Inventory_Ledger_Pachauri.xlsx
+++ b/Inventory_Ledger_Pachauri.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Inventory Ledger" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Activity Audit Log" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Security Audit Log" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -688,7 +688,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Automated Inventory Tracking, Payment Reconciliation &amp; Activity Audit Log</t>
+          <t>Authorized Inventory Tracking, Payment Reconciliation &amp; Security Audit Log</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>OPERATIONAL INSTRUCTIONS &amp; STATUS RULES</t>
+          <t>OPERATIONAL INSTRUCTIONS &amp; SECURITY PROTOCOL</t>
         </is>
       </c>
       <c r="F63" s="4" t="n"/>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="E64" s="29" t="inlineStr">
         <is>
-          <t>1. When adding a new item entry, set Status to 'Pending'.</t>
+          <t>1. Only authenticated users (Dinesh Pachauri or Mukesh Pachauri) can make changes.</t>
         </is>
       </c>
       <c r="F64" s="4" t="n"/>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="E65" s="29" t="inlineStr">
         <is>
-          <t>2. The other person acknowledges receipt by changing Status to 'Acknowledged'.</t>
+          <t>2. To modify entries, change status, or record payments, enter your Security PIN (Default: 1234).</t>
         </is>
       </c>
       <c r="F65" s="4" t="n"/>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="E66" s="29" t="inlineStr">
         <is>
-          <t>3. Record any money transferred between parties in the PAYMENT TRACKING section.</t>
+          <t>3. Every mutation automatically logs the exact timestamp and authenticated user ID.</t>
         </is>
       </c>
       <c r="F66" s="4" t="n"/>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="E67" s="29" t="inlineStr">
         <is>
-          <t>4. When a transaction or overall balance is settled, set Status to 'Cleared'.</t>
+          <t>4. When adding a new item entry, set Status to 'Pending'.</t>
         </is>
       </c>
       <c r="F67" s="4" t="n"/>
@@ -2022,7 +2022,7 @@
       <c r="C68" s="4" t="n"/>
       <c r="E68" s="29" t="inlineStr">
         <is>
-          <t>5. Every activity &amp; status update is automatically logged in the 'Activity Audit Log' tab!</t>
+          <t>5. Other authorized person acknowledges receipt by changing Status to 'Acknowledged'.</t>
         </is>
       </c>
       <c r="F68" s="4" t="n"/>
@@ -2034,7 +2034,7 @@
     <row r="69">
       <c r="E69" s="29" t="inlineStr">
         <is>
-          <t>6. Items without prices (e.g. Wrapping Sheets) can be exchanged for goods or noted in Cleared section.</t>
+          <t>6. Audit history is preserved in the 'Security Audit Log' tab.</t>
         </is>
       </c>
       <c r="F69" s="4" t="n"/>
@@ -2138,7 +2138,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PACHAURI INVENTORY ACTIVITY &amp; AUDIT TRAIL</t>
+          <t>PACHAURI INVENTORY SECURITY &amp; ACTIVITY AUDIT LOG</t>
         </is>
       </c>
     </row>
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>Performed By (Operator)</t>
+          <t>Authenticated User</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>Activity Description &amp; Details</t>
+          <t>Activity &amp; Security Audit Details</t>
         </is>
       </c>
     </row>
@@ -2230,17 +2230,17 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>System Auto</t>
+          <t>System Security</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Ledger Generated</t>
+          <t>Ledger Initialized</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Automated ledger initialized with net balance difference: Dinesh owes Mukesh ₹7,450.00</t>
+          <t>Automated ledger initialized with security PIN authentication &amp; time-stamped audit logging.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement mandatory full-screen login gate, forced password change on default 12345, and permanent shared audit log
</commit_message>
<xml_diff>
--- a/Inventory_Ledger_Pachauri.xlsx
+++ b/Inventory_Ledger_Pachauri.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Inventory Ledger" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Security Audit Log" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Shared Activity Audit Log" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -688,7 +688,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Authorized Inventory Tracking, Payment Reconciliation &amp; Security Audit Log</t>
+          <t>Mandatory Login Accounts, Password Security &amp; Permanent Shared Audit Log</t>
         </is>
       </c>
     </row>
@@ -1899,7 +1899,7 @@
     <row r="62" ht="24" customHeight="1">
       <c r="A62" s="26" t="inlineStr">
         <is>
-          <t>BALANCE RECONCILIATION &amp; INSTRUCTIONS</t>
+          <t>BALANCE RECONCILIATION &amp; SECURITY PROTOCOL</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>OPERATIONAL INSTRUCTIONS &amp; SECURITY PROTOCOL</t>
+          <t>MANDATORY LOGIN &amp; IMMUTABLE AUDIT RULES</t>
         </is>
       </c>
       <c r="F63" s="4" t="n"/>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="E64" s="29" t="inlineStr">
         <is>
-          <t>1. Only authenticated users (Dinesh Pachauri or Mukesh Pachauri) can make changes.</t>
+          <t>1. Login is mandatory. Accounts 'dinesh' &amp; 'mukesh' must authenticate to use the ledger.</t>
         </is>
       </c>
       <c r="F64" s="4" t="n"/>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="E65" s="29" t="inlineStr">
         <is>
-          <t>2. To modify entries, change status, or record payments, enter your Security PIN (Default: 1234).</t>
+          <t>2. Initial default password '12345' MUST be changed upon first login.</t>
         </is>
       </c>
       <c r="F65" s="4" t="n"/>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="E66" s="29" t="inlineStr">
         <is>
-          <t>3. Every mutation automatically logs the exact timestamp and authenticated user ID.</t>
+          <t>3. Every mutation records date, time, and logged-in user into the shared audit log.</t>
         </is>
       </c>
       <c r="F66" s="4" t="n"/>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="E67" s="29" t="inlineStr">
         <is>
-          <t>4. When adding a new item entry, set Status to 'Pending'.</t>
+          <t>4. The Shared Activity Audit Log is PERMANENT and CANNOT be deleted by anyone.</t>
         </is>
       </c>
       <c r="F67" s="4" t="n"/>
@@ -2022,7 +2022,7 @@
       <c r="C68" s="4" t="n"/>
       <c r="E68" s="29" t="inlineStr">
         <is>
-          <t>5. Other authorized person acknowledges receipt by changing Status to 'Acknowledged'.</t>
+          <t>5. Both Dinesh and Mukesh can inspect all activity logs at any time.</t>
         </is>
       </c>
       <c r="F68" s="4" t="n"/>
@@ -2034,7 +2034,7 @@
     <row r="69">
       <c r="E69" s="29" t="inlineStr">
         <is>
-          <t>6. Audit history is preserved in the 'Security Audit Log' tab.</t>
+          <t>6. Items without prices (e.g. Wrapping Sheets) are logged for inventory exchange.</t>
         </is>
       </c>
       <c r="F69" s="4" t="n"/>
@@ -2138,7 +2138,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PACHAURI INVENTORY SECURITY &amp; ACTIVITY AUDIT LOG</t>
+          <t>PACHAURI INVENTORY IMMUTABLE ACTIVITY &amp; AUDIT TRAIL</t>
         </is>
       </c>
     </row>
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>Authenticated User</t>
+          <t>Logged In User</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
@@ -2235,12 +2235,12 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Ledger Initialized</t>
+          <t>Accounts Created</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Automated ledger initialized with security PIN authentication &amp; time-stamped audit logging.</t>
+          <t>Created accounts 'dinesh' and 'mukesh' with default password '12345' (Mandatory change on first login).</t>
         </is>
       </c>
     </row>

</xml_diff>